<commit_message>
reviewed and updated confidence for some track styles
</commit_message>
<xml_diff>
--- a/playlist.xlsx
+++ b/playlist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbaune/Documents/wtf_am_i_listening/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{458EEF6D-7E3F-F340-B5FE-90B79DECBECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A3FDCC7-F39C-D749-872C-A8412575A1FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="720" yWindow="660" windowWidth="29520" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3591,6 +3591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E440"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3635,7 +3636,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -3652,7 +3653,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>15</v>
       </c>
@@ -3683,10 +3684,10 @@
         <v>22</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3703,7 +3704,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>27</v>
       </c>
@@ -3720,7 +3721,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>30</v>
       </c>
@@ -3737,7 +3738,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>33</v>
       </c>
@@ -3754,7 +3755,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>37</v>
       </c>
@@ -3771,7 +3772,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>40</v>
       </c>
@@ -3788,7 +3789,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>44</v>
       </c>
@@ -3805,7 +3806,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>47</v>
       </c>
@@ -3822,7 +3823,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>50</v>
       </c>
@@ -3839,7 +3840,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>54</v>
       </c>
@@ -3856,7 +3857,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>57</v>
       </c>
@@ -3873,7 +3874,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>60</v>
       </c>
@@ -3904,10 +3905,10 @@
         <v>66</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>67</v>
       </c>
@@ -3924,7 +3925,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>71</v>
       </c>
@@ -3941,7 +3942,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>74</v>
       </c>
@@ -3958,7 +3959,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>78</v>
       </c>
@@ -3975,7 +3976,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>81</v>
       </c>
@@ -3992,7 +3993,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>85</v>
       </c>
@@ -4009,7 +4010,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>88</v>
       </c>
@@ -4026,7 +4027,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>91</v>
       </c>
@@ -4043,7 +4044,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>95</v>
       </c>
@@ -4060,7 +4061,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>98</v>
       </c>
@@ -4077,7 +4078,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>101</v>
       </c>
@@ -4094,7 +4095,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>104</v>
       </c>
@@ -4125,10 +4126,10 @@
         <v>139</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>111</v>
       </c>
@@ -4145,7 +4146,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>114</v>
       </c>
@@ -4162,7 +4163,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>117</v>
       </c>
@@ -4179,7 +4180,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>120</v>
       </c>
@@ -4196,7 +4197,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>123</v>
       </c>
@@ -4213,7 +4214,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>126</v>
       </c>
@@ -4230,7 +4231,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>130</v>
       </c>
@@ -4247,7 +4248,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>133</v>
       </c>
@@ -4264,7 +4265,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>136</v>
       </c>
@@ -4281,7 +4282,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>140</v>
       </c>
@@ -4298,7 +4299,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>143</v>
       </c>
@@ -4315,7 +4316,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>146</v>
       </c>
@@ -4332,7 +4333,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>149</v>
       </c>
@@ -4349,7 +4350,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>152</v>
       </c>
@@ -4366,7 +4367,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>155</v>
       </c>
@@ -4383,7 +4384,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>158</v>
       </c>
@@ -4400,7 +4401,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>161</v>
       </c>
@@ -4417,7 +4418,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>165</v>
       </c>
@@ -4434,7 +4435,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>168</v>
       </c>
@@ -4451,7 +4452,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>171</v>
       </c>
@@ -4468,7 +4469,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>174</v>
       </c>
@@ -4499,10 +4500,10 @@
         <v>13</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>180</v>
       </c>
@@ -4519,7 +4520,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>180</v>
       </c>
@@ -4550,10 +4551,10 @@
         <v>8</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>185</v>
       </c>
@@ -4570,7 +4571,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>188</v>
       </c>
@@ -4598,13 +4599,13 @@
         <v>193</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>84</v>
+        <v>139</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>194</v>
       </c>
@@ -4621,7 +4622,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>195</v>
       </c>
@@ -4638,7 +4639,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>198</v>
       </c>
@@ -4669,10 +4670,10 @@
         <v>70</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>205</v>
       </c>
@@ -4689,7 +4690,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>207</v>
       </c>
@@ -4706,7 +4707,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>210</v>
       </c>
@@ -4723,7 +4724,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>212</v>
       </c>
@@ -4751,13 +4752,13 @@
         <v>217</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>13</v>
+        <v>164</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>218</v>
       </c>
@@ -4774,7 +4775,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
         <v>221</v>
       </c>
@@ -4802,13 +4803,13 @@
         <v>226</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>8</v>
+        <v>129</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>227</v>
       </c>
@@ -4825,7 +4826,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>230</v>
       </c>
@@ -4842,7 +4843,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>233</v>
       </c>
@@ -4859,7 +4860,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
         <v>236</v>
       </c>
@@ -4876,7 +4877,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>239</v>
       </c>
@@ -4893,7 +4894,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>242</v>
       </c>
@@ -4910,7 +4911,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>245</v>
       </c>
@@ -4927,7 +4928,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
         <v>246</v>
       </c>
@@ -4944,7 +4945,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
         <v>249</v>
       </c>
@@ -4961,7 +4962,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
         <v>251</v>
       </c>
@@ -4978,7 +4979,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
         <v>254</v>
       </c>
@@ -4995,7 +4996,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
         <v>257</v>
       </c>
@@ -5012,7 +5013,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
         <v>260</v>
       </c>
@@ -5029,7 +5030,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
         <v>261</v>
       </c>
@@ -5046,7 +5047,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
         <v>264</v>
       </c>
@@ -5063,7 +5064,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
         <v>267</v>
       </c>
@@ -5080,7 +5081,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
         <v>270</v>
       </c>
@@ -5097,7 +5098,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
         <v>273</v>
       </c>
@@ -5114,7 +5115,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
         <v>276</v>
       </c>
@@ -5131,7 +5132,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
         <v>277</v>
       </c>
@@ -5148,7 +5149,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
         <v>280</v>
       </c>
@@ -5176,13 +5177,13 @@
         <v>286</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>283</v>
+        <v>8</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
         <v>287</v>
       </c>
@@ -5199,7 +5200,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
         <v>290</v>
       </c>
@@ -5216,7 +5217,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
         <v>292</v>
       </c>
@@ -5233,7 +5234,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
         <v>295</v>
       </c>
@@ -5264,7 +5265,7 @@
         <v>94</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.2">
@@ -5284,7 +5285,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A100" s="2" t="s">
         <v>304</v>
       </c>
@@ -5301,7 +5302,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A101" s="2" t="s">
         <v>306</v>
       </c>
@@ -5318,7 +5319,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A102" s="2" t="s">
         <v>309</v>
       </c>
@@ -5335,7 +5336,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A103" s="2" t="s">
         <v>312</v>
       </c>
@@ -5369,7 +5370,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A105" s="2" t="s">
         <v>318</v>
       </c>
@@ -5386,7 +5387,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
         <v>321</v>
       </c>
@@ -5403,7 +5404,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A107" s="2" t="s">
         <v>324</v>
       </c>
@@ -5431,10 +5432,10 @@
         <v>329</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.2">
@@ -5454,7 +5455,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A110" s="2" t="s">
         <v>333</v>
       </c>
@@ -5488,7 +5489,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A112" s="2" t="s">
         <v>340</v>
       </c>
@@ -5522,7 +5523,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A114" s="2" t="s">
         <v>346</v>
       </c>
@@ -5539,7 +5540,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A115" s="2" t="s">
         <v>350</v>
       </c>
@@ -5556,7 +5557,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A116" s="2" t="s">
         <v>351</v>
       </c>
@@ -5573,7 +5574,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A117" s="2" t="s">
         <v>353</v>
       </c>
@@ -5604,10 +5605,10 @@
         <v>8</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A119" s="2" t="s">
         <v>359</v>
       </c>
@@ -5638,10 +5639,10 @@
         <v>8</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A121" s="2" t="s">
         <v>365</v>
       </c>
@@ -5658,7 +5659,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A122" s="2" t="s">
         <v>368</v>
       </c>
@@ -5692,7 +5693,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A124" s="2" t="s">
         <v>374</v>
       </c>
@@ -5709,7 +5710,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A125" s="2" t="s">
         <v>375</v>
       </c>
@@ -5737,13 +5738,13 @@
         <v>379</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="E126" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A127" s="2" t="s">
         <v>380</v>
       </c>
@@ -5774,10 +5775,10 @@
         <v>8</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A129" s="2" t="s">
         <v>385</v>
       </c>
@@ -5794,7 +5795,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A130" s="2" t="s">
         <v>388</v>
       </c>
@@ -5811,7 +5812,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A131" s="2" t="s">
         <v>390</v>
       </c>
@@ -5828,7 +5829,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A132" s="2" t="s">
         <v>393</v>
       </c>
@@ -5845,7 +5846,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A133" s="2" t="s">
         <v>396</v>
       </c>
@@ -5862,7 +5863,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A134" s="2" t="s">
         <v>399</v>
       </c>
@@ -5879,7 +5880,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A135" s="2" t="s">
         <v>402</v>
       </c>
@@ -5913,7 +5914,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A137" s="2" t="s">
         <v>408</v>
       </c>
@@ -5930,7 +5931,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A138" s="2" t="s">
         <v>410</v>
       </c>
@@ -5947,7 +5948,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A139" s="2" t="s">
         <v>413</v>
       </c>
@@ -5964,7 +5965,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A140" s="2" t="s">
         <v>416</v>
       </c>
@@ -5995,7 +5996,7 @@
         <v>8</v>
       </c>
       <c r="E141" s="2" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.2">
@@ -6012,10 +6013,10 @@
         <v>94</v>
       </c>
       <c r="E142" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A143" s="2" t="s">
         <v>424</v>
       </c>
@@ -6032,7 +6033,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A144" s="2" t="s">
         <v>426</v>
       </c>
@@ -6049,7 +6050,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A145" s="2" t="s">
         <v>429</v>
       </c>
@@ -6066,7 +6067,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A146" s="2" t="s">
         <v>430</v>
       </c>
@@ -6083,7 +6084,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A147" s="2" t="s">
         <v>433</v>
       </c>
@@ -6100,7 +6101,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A148" s="2" t="s">
         <v>436</v>
       </c>
@@ -6128,10 +6129,10 @@
         <v>441</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>8</v>
+        <v>94</v>
       </c>
       <c r="E149" s="2" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.2">
@@ -6151,7 +6152,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A151" s="2" t="s">
         <v>445</v>
       </c>
@@ -6182,7 +6183,7 @@
         <v>18</v>
       </c>
       <c r="E152" s="2" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.2">
@@ -6219,7 +6220,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A155" s="2" t="s">
         <v>457</v>
       </c>
@@ -6236,7 +6237,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A156" s="2" t="s">
         <v>459</v>
       </c>
@@ -6284,10 +6285,10 @@
         <v>139</v>
       </c>
       <c r="E158" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A159" s="2" t="s">
         <v>467</v>
       </c>
@@ -6304,7 +6305,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A160" s="2" t="s">
         <v>470</v>
       </c>
@@ -6335,10 +6336,10 @@
         <v>66</v>
       </c>
       <c r="E161" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A162" s="2" t="s">
         <v>475</v>
       </c>
@@ -6355,7 +6356,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A163" s="2" t="s">
         <v>478</v>
       </c>
@@ -6372,7 +6373,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A164" s="2" t="s">
         <v>480</v>
       </c>
@@ -6389,7 +6390,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A165" s="2" t="s">
         <v>483</v>
       </c>
@@ -6406,7 +6407,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A166" s="2" t="s">
         <v>485</v>
       </c>
@@ -6423,7 +6424,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A167" s="2" t="s">
         <v>486</v>
       </c>
@@ -6440,7 +6441,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A168" s="2" t="s">
         <v>488</v>
       </c>
@@ -6457,7 +6458,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A169" s="2" t="s">
         <v>490</v>
       </c>
@@ -6474,7 +6475,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A170" s="2" t="s">
         <v>492</v>
       </c>
@@ -6491,7 +6492,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A171" s="2" t="s">
         <v>495</v>
       </c>
@@ -6508,7 +6509,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A172" s="2" t="s">
         <v>498</v>
       </c>
@@ -6539,7 +6540,7 @@
         <v>22</v>
       </c>
       <c r="E173" s="2" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.2">
@@ -6559,7 +6560,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A175" s="2" t="s">
         <v>507</v>
       </c>
@@ -6593,7 +6594,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A177" s="2" t="s">
         <v>513</v>
       </c>
@@ -6610,7 +6611,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A178" s="2" t="s">
         <v>515</v>
       </c>
@@ -6627,7 +6628,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A179" s="2" t="s">
         <v>518</v>
       </c>
@@ -6644,7 +6645,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A180" s="2" t="s">
         <v>521</v>
       </c>
@@ -6695,7 +6696,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A183" s="2" t="s">
         <v>529</v>
       </c>
@@ -6712,7 +6713,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A184" s="2" t="s">
         <v>532</v>
       </c>
@@ -6729,7 +6730,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A185" s="2" t="s">
         <v>534</v>
       </c>
@@ -6746,7 +6747,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A186" s="2" t="s">
         <v>536</v>
       </c>
@@ -6763,7 +6764,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A187" s="2" t="s">
         <v>537</v>
       </c>
@@ -6780,7 +6781,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A188" s="2" t="s">
         <v>540</v>
       </c>
@@ -6797,7 +6798,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A189" s="2" t="s">
         <v>543</v>
       </c>
@@ -6814,7 +6815,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A190" s="2" t="s">
         <v>546</v>
       </c>
@@ -6831,7 +6832,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A191" s="2" t="s">
         <v>549</v>
       </c>
@@ -6848,7 +6849,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A192" s="2" t="s">
         <v>552</v>
       </c>
@@ -6865,7 +6866,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A193" s="2" t="s">
         <v>555</v>
       </c>
@@ -6882,7 +6883,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A194" s="2" t="s">
         <v>557</v>
       </c>
@@ -6899,7 +6900,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A195" s="2" t="s">
         <v>559</v>
       </c>
@@ -6933,7 +6934,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A197" s="2" t="s">
         <v>563</v>
       </c>
@@ -6967,7 +6968,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A199" s="2" t="s">
         <v>568</v>
       </c>
@@ -6984,7 +6985,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A200" s="2" t="s">
         <v>571</v>
       </c>
@@ -7015,10 +7016,10 @@
         <v>164</v>
       </c>
       <c r="E201" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A202" s="2" t="s">
         <v>576</v>
       </c>
@@ -7035,7 +7036,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A203" s="2" t="s">
         <v>579</v>
       </c>
@@ -7052,7 +7053,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A204" s="2" t="s">
         <v>582</v>
       </c>
@@ -7086,7 +7087,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A206" s="2" t="s">
         <v>587</v>
       </c>
@@ -7117,7 +7118,7 @@
         <v>592</v>
       </c>
       <c r="E207" s="2" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.2">
@@ -7134,10 +7135,10 @@
         <v>592</v>
       </c>
       <c r="E208" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A209" s="2" t="s">
         <v>596</v>
       </c>
@@ -7154,7 +7155,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A210" s="2" t="s">
         <v>597</v>
       </c>
@@ -7171,7 +7172,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A211" s="2" t="s">
         <v>600</v>
       </c>
@@ -7188,7 +7189,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A212" s="2" t="s">
         <v>603</v>
       </c>
@@ -7205,7 +7206,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A213" s="2" t="s">
         <v>606</v>
       </c>
@@ -7222,7 +7223,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A214" s="2" t="s">
         <v>608</v>
       </c>
@@ -7239,7 +7240,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A215" s="2" t="s">
         <v>611</v>
       </c>
@@ -7256,7 +7257,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A216" s="2" t="s">
         <v>614</v>
       </c>
@@ -7273,7 +7274,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A217" s="2" t="s">
         <v>617</v>
       </c>
@@ -7307,7 +7308,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A219" s="2" t="s">
         <v>623</v>
       </c>
@@ -7324,7 +7325,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A220" s="2" t="s">
         <v>625</v>
       </c>
@@ -7341,7 +7342,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A221" s="2" t="s">
         <v>628</v>
       </c>
@@ -7358,7 +7359,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A222" s="2" t="s">
         <v>631</v>
       </c>
@@ -7375,7 +7376,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A223" s="2" t="s">
         <v>632</v>
       </c>
@@ -7392,7 +7393,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A224" s="2" t="s">
         <v>635</v>
       </c>
@@ -7409,7 +7410,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A225" s="2" t="s">
         <v>637</v>
       </c>
@@ -7426,7 +7427,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A226" s="2" t="s">
         <v>640</v>
       </c>
@@ -7443,7 +7444,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A227" s="2" t="s">
         <v>641</v>
       </c>
@@ -7471,7 +7472,7 @@
         <v>646</v>
       </c>
       <c r="D228" s="2" t="s">
-        <v>110</v>
+        <v>8</v>
       </c>
       <c r="E228" s="2" t="s">
         <v>26</v>
@@ -7491,7 +7492,7 @@
         <v>592</v>
       </c>
       <c r="E229" s="2" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
     </row>
     <row r="230" spans="1:5" x14ac:dyDescent="0.2">
@@ -7511,7 +7512,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A231" s="2" t="s">
         <v>653</v>
       </c>
@@ -7528,7 +7529,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A232" s="2" t="s">
         <v>656</v>
       </c>
@@ -7545,7 +7546,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A233" s="2" t="s">
         <v>657</v>
       </c>
@@ -7562,7 +7563,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A234" s="2" t="s">
         <v>658</v>
       </c>
@@ -7579,7 +7580,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A235" s="2" t="s">
         <v>659</v>
       </c>
@@ -7596,7 +7597,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A236" s="2" t="s">
         <v>662</v>
       </c>
@@ -7613,7 +7614,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A237" s="2" t="s">
         <v>665</v>
       </c>
@@ -7644,7 +7645,7 @@
         <v>18</v>
       </c>
       <c r="E238" s="2" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
     <row r="239" spans="1:5" x14ac:dyDescent="0.2">
@@ -7664,7 +7665,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A240" s="2" t="s">
         <v>674</v>
       </c>
@@ -7681,7 +7682,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A241" s="2" t="s">
         <v>677</v>
       </c>
@@ -7698,7 +7699,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A242" s="2" t="s">
         <v>679</v>
       </c>
@@ -7715,7 +7716,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A243" s="2" t="s">
         <v>682</v>
       </c>
@@ -7732,7 +7733,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A244" s="2" t="s">
         <v>685</v>
       </c>
@@ -7749,7 +7750,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A245" s="2" t="s">
         <v>688</v>
       </c>
@@ -7766,7 +7767,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A246" s="2" t="s">
         <v>691</v>
       </c>
@@ -7783,7 +7784,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A247" s="2" t="s">
         <v>694</v>
       </c>
@@ -7800,7 +7801,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A248" s="2" t="s">
         <v>697</v>
       </c>
@@ -7831,10 +7832,10 @@
         <v>349</v>
       </c>
       <c r="E249" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="250" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A250" s="2" t="s">
         <v>702</v>
       </c>
@@ -7851,7 +7852,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A251" s="2" t="s">
         <v>704</v>
       </c>
@@ -7868,7 +7869,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A252" s="2" t="s">
         <v>707</v>
       </c>
@@ -7899,10 +7900,10 @@
         <v>94</v>
       </c>
       <c r="E253" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="254" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A254" s="2" t="s">
         <v>713</v>
       </c>
@@ -7919,7 +7920,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A255" s="2" t="s">
         <v>716</v>
       </c>
@@ -7936,7 +7937,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A256" s="2" t="s">
         <v>718</v>
       </c>
@@ -7967,10 +7968,10 @@
         <v>8</v>
       </c>
       <c r="E257" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="258" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A258" s="2" t="s">
         <v>723</v>
       </c>
@@ -8001,10 +8002,10 @@
         <v>22</v>
       </c>
       <c r="E259" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="260" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A260" s="2" t="s">
         <v>727</v>
       </c>
@@ -8021,7 +8022,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A261" s="2" t="s">
         <v>729</v>
       </c>
@@ -8038,7 +8039,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A262" s="2" t="s">
         <v>731</v>
       </c>
@@ -8055,7 +8056,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A263" s="2" t="s">
         <v>732</v>
       </c>
@@ -8072,7 +8073,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A264" s="2" t="s">
         <v>735</v>
       </c>
@@ -8103,10 +8104,10 @@
         <v>22</v>
       </c>
       <c r="E265" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="266" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A266" s="2" t="s">
         <v>741</v>
       </c>
@@ -8123,7 +8124,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A267" s="2" t="s">
         <v>744</v>
       </c>
@@ -8140,7 +8141,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A268" s="2" t="s">
         <v>747</v>
       </c>
@@ -8174,7 +8175,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A270" s="2" t="s">
         <v>751</v>
       </c>
@@ -8191,7 +8192,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A271" s="2" t="s">
         <v>754</v>
       </c>
@@ -8222,7 +8223,7 @@
         <v>94</v>
       </c>
       <c r="E272" s="2" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
     <row r="273" spans="1:5" x14ac:dyDescent="0.2">
@@ -8239,7 +8240,7 @@
         <v>94</v>
       </c>
       <c r="E273" s="2" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
     </row>
     <row r="274" spans="1:5" x14ac:dyDescent="0.2">
@@ -8259,7 +8260,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A275" s="2" t="s">
         <v>766</v>
       </c>
@@ -8276,7 +8277,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A276" s="2" t="s">
         <v>768</v>
       </c>
@@ -8293,7 +8294,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A277" s="2" t="s">
         <v>770</v>
       </c>
@@ -8310,7 +8311,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A278" s="2" t="s">
         <v>772</v>
       </c>
@@ -8327,7 +8328,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A279" s="2" t="s">
         <v>775</v>
       </c>
@@ -8344,7 +8345,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A280" s="2" t="s">
         <v>778</v>
       </c>
@@ -8361,7 +8362,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A281" s="2" t="s">
         <v>781</v>
       </c>
@@ -8378,7 +8379,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A282" s="2" t="s">
         <v>782</v>
       </c>
@@ -8395,7 +8396,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A283" s="2" t="s">
         <v>785</v>
       </c>
@@ -8412,7 +8413,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A284" s="2" t="s">
         <v>788</v>
       </c>
@@ -8429,7 +8430,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A285" s="2" t="s">
         <v>791</v>
       </c>
@@ -8446,7 +8447,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A286" s="2" t="s">
         <v>794</v>
       </c>
@@ -8463,7 +8464,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A287" s="2" t="s">
         <v>797</v>
       </c>
@@ -8497,7 +8498,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A289" s="2" t="s">
         <v>802</v>
       </c>
@@ -8514,7 +8515,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A290" s="2" t="s">
         <v>803</v>
       </c>
@@ -8531,7 +8532,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A291" s="2" t="s">
         <v>804</v>
       </c>
@@ -8548,7 +8549,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A292" s="2" t="s">
         <v>807</v>
       </c>
@@ -8565,7 +8566,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A293" s="2" t="s">
         <v>810</v>
       </c>
@@ -8582,7 +8583,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A294" s="2" t="s">
         <v>812</v>
       </c>
@@ -8599,7 +8600,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A295" s="2" t="s">
         <v>815</v>
       </c>
@@ -8616,7 +8617,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A296" s="2" t="s">
         <v>818</v>
       </c>
@@ -8633,7 +8634,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A297" s="2" t="s">
         <v>821</v>
       </c>
@@ -8667,7 +8668,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A299" s="2" t="s">
         <v>825</v>
       </c>
@@ -8698,7 +8699,7 @@
         <v>18</v>
       </c>
       <c r="E300" s="2" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
     </row>
     <row r="301" spans="1:5" x14ac:dyDescent="0.2">
@@ -8715,10 +8716,10 @@
         <v>18</v>
       </c>
       <c r="E301" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="302" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A302" s="2" t="s">
         <v>830</v>
       </c>
@@ -8735,7 +8736,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A303" s="2" t="s">
         <v>833</v>
       </c>
@@ -8766,10 +8767,10 @@
         <v>13</v>
       </c>
       <c r="E304" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="305" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A305" s="2" t="s">
         <v>838</v>
       </c>
@@ -8786,7 +8787,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A306" s="2" t="s">
         <v>841</v>
       </c>
@@ -8803,7 +8804,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A307" s="2" t="s">
         <v>843</v>
       </c>
@@ -8820,7 +8821,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A308" s="2" t="s">
         <v>846</v>
       </c>
@@ -8837,7 +8838,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A309" s="2" t="s">
         <v>847</v>
       </c>
@@ -8854,7 +8855,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A310" s="2" t="s">
         <v>850</v>
       </c>
@@ -8871,7 +8872,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A311" s="2" t="s">
         <v>853</v>
       </c>
@@ -8888,7 +8889,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A312" s="2" t="s">
         <v>856</v>
       </c>
@@ -8905,7 +8906,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A313" s="2" t="s">
         <v>859</v>
       </c>
@@ -8922,7 +8923,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A314" s="2" t="s">
         <v>862</v>
       </c>
@@ -8939,7 +8940,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A315" s="2" t="s">
         <v>865</v>
       </c>
@@ -8956,7 +8957,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="316" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A316" s="2" t="s">
         <v>868</v>
       </c>
@@ -8973,7 +8974,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A317" s="2" t="s">
         <v>870</v>
       </c>
@@ -8990,7 +8991,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="318" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A318" s="2" t="s">
         <v>871</v>
       </c>
@@ -9007,7 +9008,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="319" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A319" s="2" t="s">
         <v>873</v>
       </c>
@@ -9024,7 +9025,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="320" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A320" s="2" t="s">
         <v>875</v>
       </c>
@@ -9041,7 +9042,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A321" s="2" t="s">
         <v>876</v>
       </c>
@@ -9058,7 +9059,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A322" s="2" t="s">
         <v>879</v>
       </c>
@@ -9075,7 +9076,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A323" s="2" t="s">
         <v>882</v>
       </c>
@@ -9092,7 +9093,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A324" s="2" t="s">
         <v>885</v>
       </c>
@@ -9109,7 +9110,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="325" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A325" s="2" t="s">
         <v>887</v>
       </c>
@@ -9126,7 +9127,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A326" s="2" t="s">
         <v>888</v>
       </c>
@@ -9143,7 +9144,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A327" s="2" t="s">
         <v>891</v>
       </c>
@@ -9160,7 +9161,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="328" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A328" s="2" t="s">
         <v>894</v>
       </c>
@@ -9177,7 +9178,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="329" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A329" s="2" t="s">
         <v>897</v>
       </c>
@@ -9194,7 +9195,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="330" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A330" s="2" t="s">
         <v>900</v>
       </c>
@@ -9211,7 +9212,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A331" s="2" t="s">
         <v>903</v>
       </c>
@@ -9228,7 +9229,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A332" s="2" t="s">
         <v>905</v>
       </c>
@@ -9245,7 +9246,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A333" s="2" t="s">
         <v>908</v>
       </c>
@@ -9262,7 +9263,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="334" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A334" s="2" t="s">
         <v>911</v>
       </c>
@@ -9296,7 +9297,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A336" s="2" t="s">
         <v>332</v>
       </c>
@@ -9313,7 +9314,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A337" s="2" t="s">
         <v>916</v>
       </c>
@@ -9330,7 +9331,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A338" s="2" t="s">
         <v>918</v>
       </c>
@@ -9347,7 +9348,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="339" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A339" s="2" t="s">
         <v>921</v>
       </c>
@@ -9364,7 +9365,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A340" s="2" t="s">
         <v>923</v>
       </c>
@@ -9381,7 +9382,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A341" s="2" t="s">
         <v>927</v>
       </c>
@@ -9398,7 +9399,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A342" s="2" t="s">
         <v>930</v>
       </c>
@@ -9415,7 +9416,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A343" s="2" t="s">
         <v>934</v>
       </c>
@@ -9432,7 +9433,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A344" s="2" t="s">
         <v>937</v>
       </c>
@@ -9449,7 +9450,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A345" s="2" t="s">
         <v>939</v>
       </c>
@@ -9466,7 +9467,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A346" s="2" t="s">
         <v>943</v>
       </c>
@@ -9483,7 +9484,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A347" s="2" t="s">
         <v>946</v>
       </c>
@@ -9500,7 +9501,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A348" s="2" t="s">
         <v>949</v>
       </c>
@@ -9517,7 +9518,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="349" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A349" s="2" t="s">
         <v>952</v>
       </c>
@@ -9534,7 +9535,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A350" s="2" t="s">
         <v>953</v>
       </c>
@@ -9551,7 +9552,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="351" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A351" s="2" t="s">
         <v>956</v>
       </c>
@@ -9568,7 +9569,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="352" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A352" s="2" t="s">
         <v>959</v>
       </c>
@@ -9585,7 +9586,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="353" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A353" s="2" t="s">
         <v>962</v>
       </c>
@@ -9602,7 +9603,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="354" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A354" s="2" t="s">
         <v>965</v>
       </c>
@@ -9619,7 +9620,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="355" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A355" s="2" t="s">
         <v>968</v>
       </c>
@@ -9636,7 +9637,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="356" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A356" s="2" t="s">
         <v>971</v>
       </c>
@@ -9653,7 +9654,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="357" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A357" s="2" t="s">
         <v>974</v>
       </c>
@@ -9670,7 +9671,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="358" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A358" s="2" t="s">
         <v>977</v>
       </c>
@@ -9687,7 +9688,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="359" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A359" s="2" t="s">
         <v>657</v>
       </c>
@@ -9704,7 +9705,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="360" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A360" s="2" t="s">
         <v>205</v>
       </c>
@@ -9721,7 +9722,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="361" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A361" s="2" t="s">
         <v>980</v>
       </c>
@@ -9738,7 +9739,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="362" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A362" s="2" t="s">
         <v>981</v>
       </c>
@@ -9755,7 +9756,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="363" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A363" s="2" t="s">
         <v>982</v>
       </c>
@@ -9772,7 +9773,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="364" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A364" s="2" t="s">
         <v>374</v>
       </c>
@@ -9789,7 +9790,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="365" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A365" s="2" t="s">
         <v>983</v>
       </c>
@@ -9806,7 +9807,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="366" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A366" s="2" t="s">
         <v>984</v>
       </c>
@@ -9823,7 +9824,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="367" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A367" s="2" t="s">
         <v>276</v>
       </c>
@@ -9840,7 +9841,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="368" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A368" s="2" t="s">
         <v>985</v>
       </c>
@@ -9857,7 +9858,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="369" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A369" s="2" t="s">
         <v>161</v>
       </c>
@@ -9874,7 +9875,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="370" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A370" s="2" t="s">
         <v>986</v>
       </c>
@@ -9891,7 +9892,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="371" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A371" s="2" t="s">
         <v>987</v>
       </c>
@@ -9908,7 +9909,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="372" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A372" s="2" t="s">
         <v>988</v>
       </c>
@@ -9925,7 +9926,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="373" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A373" s="2" t="s">
         <v>989</v>
       </c>
@@ -9942,7 +9943,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="374" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A374" s="2" t="s">
         <v>802</v>
       </c>
@@ -9959,7 +9960,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="375" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A375" s="2" t="s">
         <v>781</v>
       </c>
@@ -9976,7 +9977,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="376" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A376" s="2" t="s">
         <v>723</v>
       </c>
@@ -9993,7 +9994,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="377" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A377" s="2" t="s">
         <v>990</v>
       </c>
@@ -10010,7 +10011,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="378" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A378" s="2" t="s">
         <v>846</v>
       </c>
@@ -10027,7 +10028,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="379" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A379" s="2" t="s">
         <v>731</v>
       </c>
@@ -10044,7 +10045,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="380" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A380" s="2" t="s">
         <v>375</v>
       </c>
@@ -10061,7 +10062,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="381" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="381" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A381" s="2" t="s">
         <v>640</v>
       </c>
@@ -10078,7 +10079,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="382" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="382" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A382" s="2" t="s">
         <v>991</v>
       </c>
@@ -10095,7 +10096,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="383" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="383" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A383" s="2" t="s">
         <v>992</v>
       </c>
@@ -10112,7 +10113,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="384" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="384" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A384" s="2" t="s">
         <v>993</v>
       </c>
@@ -10129,7 +10130,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="385" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="385" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A385" s="2" t="s">
         <v>994</v>
       </c>
@@ -10146,7 +10147,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="386" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="386" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A386" s="2" t="s">
         <v>995</v>
       </c>
@@ -10163,7 +10164,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="387" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="387" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A387" s="2" t="s">
         <v>631</v>
       </c>
@@ -10180,7 +10181,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="388" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="388" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A388" s="2" t="s">
         <v>513</v>
       </c>
@@ -10197,7 +10198,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="389" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="389" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A389" s="2" t="s">
         <v>996</v>
       </c>
@@ -10214,7 +10215,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="390" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="390" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A390" s="2" t="s">
         <v>997</v>
       </c>
@@ -10231,7 +10232,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="391" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="391" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A391" s="2" t="s">
         <v>998</v>
       </c>
@@ -10248,7 +10249,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="392" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="392" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A392" s="2" t="s">
         <v>999</v>
       </c>
@@ -10265,7 +10266,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="393" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="393" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A393" s="2" t="s">
         <v>1000</v>
       </c>
@@ -10282,7 +10283,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="394" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="394" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A394" s="2" t="s">
         <v>1001</v>
       </c>
@@ -10299,7 +10300,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="395" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="395" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A395" s="2" t="s">
         <v>1002</v>
       </c>
@@ -10316,7 +10317,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="396" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="396" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A396" s="2" t="s">
         <v>1003</v>
       </c>
@@ -10333,7 +10334,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="397" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="397" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A397" s="2" t="s">
         <v>1004</v>
       </c>
@@ -10350,7 +10351,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="398" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="398" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A398" s="2" t="s">
         <v>1005</v>
       </c>
@@ -10367,7 +10368,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="399" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="399" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A399" s="2" t="s">
         <v>716</v>
       </c>
@@ -10384,7 +10385,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="400" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="400" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A400" s="2" t="s">
         <v>1006</v>
       </c>
@@ -10401,7 +10402,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="401" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="401" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A401" s="2" t="s">
         <v>1007</v>
       </c>
@@ -10418,7 +10419,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="402" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="402" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A402" s="2" t="s">
         <v>1008</v>
       </c>
@@ -10435,7 +10436,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="403" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="403" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A403" s="2" t="s">
         <v>1009</v>
       </c>
@@ -10452,7 +10453,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="404" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="404" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A404" s="2" t="s">
         <v>1010</v>
       </c>
@@ -10469,7 +10470,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="405" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="405" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A405" s="2" t="s">
         <v>1011</v>
       </c>
@@ -10486,7 +10487,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="406" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="406" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A406" s="2" t="s">
         <v>1012</v>
       </c>
@@ -10503,7 +10504,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="407" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="407" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A407" s="2" t="s">
         <v>1013</v>
       </c>
@@ -10520,7 +10521,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="408" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="408" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A408" s="2" t="s">
         <v>1014</v>
       </c>
@@ -10537,7 +10538,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="409" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="409" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A409" s="2" t="s">
         <v>1015</v>
       </c>
@@ -10554,7 +10555,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="410" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="410" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A410" s="2" t="s">
         <v>1016</v>
       </c>
@@ -10571,7 +10572,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="411" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="411" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A411" s="2" t="s">
         <v>1017</v>
       </c>
@@ -10588,7 +10589,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="412" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="412" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A412" s="2" t="s">
         <v>1018</v>
       </c>
@@ -10605,7 +10606,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="413" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="413" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A413" s="2" t="s">
         <v>658</v>
       </c>
@@ -10622,7 +10623,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="414" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="414" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A414" s="2" t="s">
         <v>194</v>
       </c>
@@ -10639,7 +10640,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="415" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="415" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A415" s="2" t="s">
         <v>1019</v>
       </c>
@@ -10656,7 +10657,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="416" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="416" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A416" s="2" t="s">
         <v>1020</v>
       </c>
@@ -10673,7 +10674,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="417" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="417" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A417" s="2" t="s">
         <v>1021</v>
       </c>
@@ -10690,7 +10691,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="418" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="418" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A418" s="2" t="s">
         <v>1022</v>
       </c>
@@ -10707,7 +10708,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="419" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="419" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A419" s="2" t="s">
         <v>1023</v>
       </c>
@@ -10724,7 +10725,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="420" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="420" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A420" s="2" t="s">
         <v>1008</v>
       </c>
@@ -10741,7 +10742,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="421" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="421" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A421" s="2" t="s">
         <v>1024</v>
       </c>
@@ -10758,7 +10759,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="422" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="422" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A422" s="2" t="s">
         <v>1025</v>
       </c>
@@ -10775,7 +10776,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="423" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="423" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A423" s="2" t="s">
         <v>180</v>
       </c>
@@ -10792,7 +10793,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="424" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="424" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A424" s="2" t="s">
         <v>1026</v>
       </c>
@@ -10809,7 +10810,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="425" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="425" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A425" s="2" t="s">
         <v>1013</v>
       </c>
@@ -10826,7 +10827,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="426" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="426" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A426" s="2" t="s">
         <v>1027</v>
       </c>
@@ -10843,7 +10844,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="427" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="427" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A427" s="2" t="s">
         <v>1028</v>
       </c>
@@ -10860,7 +10861,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="428" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="428" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A428" s="2" t="s">
         <v>1029</v>
       </c>
@@ -10877,7 +10878,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="429" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="429" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A429" s="2" t="s">
         <v>1030</v>
       </c>
@@ -10894,7 +10895,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="430" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="430" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A430" s="2" t="s">
         <v>1018</v>
       </c>
@@ -10911,7 +10912,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="431" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="431" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A431" s="2" t="s">
         <v>658</v>
       </c>
@@ -10928,7 +10929,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="432" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="432" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A432" s="2" t="s">
         <v>194</v>
       </c>
@@ -10945,7 +10946,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="433" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="433" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A433" s="2" t="s">
         <v>1019</v>
       </c>
@@ -10962,7 +10963,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="434" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="434" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A434" s="2" t="s">
         <v>495</v>
       </c>
@@ -10979,7 +10980,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="435" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="435" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A435" s="2" t="s">
         <v>1031</v>
       </c>
@@ -10996,7 +10997,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="436" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="436" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A436" s="2" t="s">
         <v>916</v>
       </c>
@@ -11013,7 +11014,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="437" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="437" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A437" s="2" t="s">
         <v>1034</v>
       </c>
@@ -11030,7 +11031,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="438" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="438" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A438" s="2" t="s">
         <v>1035</v>
       </c>
@@ -11047,7 +11048,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="439" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="439" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A439" s="2" t="s">
         <v>351</v>
       </c>
@@ -11064,7 +11065,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="440" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="440" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A440" s="2" t="s">
         <v>1036</v>
       </c>
@@ -11082,7 +11083,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E440" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:E440" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Best guess"/>
+        <filter val="Likely"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Certainty" error="Pick Confident, Likely or Best guess, or leave it empty." sqref="E2:E10000" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Confident,Likely,Best guess"</formula1>

</xml_diff>